<commit_message>
docs(hw01): align the AI-02 disclosure with the report
Record the remaining fan defects, verified AI errors, and self-assessment, and state that Cursor formatted the observed results into the report, workbook, and issues.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/HW01/HW01_Test_Workbook.xlsx
+++ b/HW01/HW01_Test_Workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Test Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Test Cases" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Checklist" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Defects" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -896,7 +896,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>[To be written after execution: which tests failed, open defects, residual risks, recommendation.]</t>
+          <t>Executed 9 of 15 tests on 27/09/2026: 4 PASS, 5 FAIL, 6 NOT RUN. Five defects are open (DF-01 to DF-05). DF-04 (gear grinds, oscillation does not resume) and DF-05 (finger reaches a blade through the rear guard) are High. DF-02 and DF-03 have no video yet. Residual risk: TC-02, TC-05, TC-13 and TC-15 are not run, so start-up, coast-down, stability and the 60-minute run are still unknown.</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1219,12 @@
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. Turning the knob in one movement from 1 to 3, the motor clicks one beat each time the pointer passes the midpoint between two marks. When the knob stops on a mark, the speed matches that mark.</t>
         </is>
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I8" s="8" t="inlineStr">
@@ -1237,9 +1237,17 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K8" s="8" t="inlineStr"/>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
       <c r="L8" s="8" t="inlineStr"/>
-      <c r="M8" s="8" t="inlineStr"/>
+      <c r="M8" s="8" t="inlineStr">
+        <is>
+          <t>DF-02 https://github.com/Toanapr/Homework/issues/2</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1331,12 +1339,12 @@
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. When the knob is left between two speed marks, the fan switches off.</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
@@ -1349,9 +1357,21 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K10" s="8" t="inlineStr"/>
-      <c r="L10" s="8" t="inlineStr"/>
-      <c r="M10" s="8" t="inlineStr"/>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/k_u6U1VcS8w</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="inlineStr">
+        <is>
+          <t>DF-01 https://github.com/Toanapr/Homework/issues/1</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1388,12 +1408,12 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. Turning past 3 moves the knob to 0 and the fan switches off. Turning onward from 0 moves the knob to the next marked position. The speed matches the mark.</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I11" s="8" t="inlineStr">
@@ -1406,8 +1426,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" s="8" t="inlineStr"/>
-      <c r="L11" s="8" t="inlineStr"/>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/ttXP6ScmhF8</t>
+        </is>
+      </c>
       <c r="M11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
@@ -1446,12 +1474,12 @@
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. Switching oscillation off while the head is sweeping, the head sweeps more than one extra turn before it stops.</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
@@ -1464,9 +1492,17 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K12" s="8" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
       <c r="L12" s="8" t="inlineStr"/>
-      <c r="M12" s="8" t="inlineStr"/>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>DF-03 https://github.com/Toanapr/Homework/issues/3</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1502,12 +1538,12 @@
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. The head keeps sweeping at speeds 1, 2 and 3, with no sticking or grinding.</t>
         </is>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I13" s="8" t="inlineStr">
@@ -1520,8 +1556,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="K13" s="8" t="inlineStr"/>
-      <c r="L13" s="8" t="inlineStr"/>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/Kd-fHpxxTQ0</t>
+        </is>
+      </c>
       <c r="M13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
@@ -1559,12 +1603,12 @@
       </c>
       <c r="G14" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. Setting oscillation while the fan is off does not start it. After turning to speed 1, the fan runs and oscillates.</t>
         </is>
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I14" s="8" t="inlineStr">
@@ -1577,8 +1621,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="8" t="inlineStr"/>
-      <c r="L14" s="8" t="inlineStr"/>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/UN6RFUItYyA</t>
+        </is>
+      </c>
       <c r="M14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1615,12 +1667,12 @@
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. Holding the head still for 2 seconds while it is oscillating, the gears grind. After release the head stays still and oscillation does not resume.</t>
         </is>
       </c>
       <c r="H15" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -1633,9 +1685,17 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K15" s="8" t="inlineStr"/>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
       <c r="L15" s="8" t="inlineStr"/>
-      <c r="M15" s="8" t="inlineStr"/>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>DF-04 https://github.com/Toanapr/Homework/issues/4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1671,12 +1731,12 @@
       </c>
       <c r="G16" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. With the knob at 2, the fan restarts at speed 2 when power returns. With the knob at 0, it stays off.</t>
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -1689,8 +1749,16 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="K16" s="8" t="inlineStr"/>
-      <c r="L16" s="8" t="inlineStr"/>
+      <c r="K16" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="L16" s="8" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/2LpDTG9UcTU</t>
+        </is>
+      </c>
       <c r="M16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1784,12 +1852,12 @@
       </c>
       <c r="G18" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>27/09/2026. With the fan unplugged, a fingertip cannot touch a blade through the front guard. Through the rear guard a fingertip can touch a blade.</t>
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr">
@@ -1802,9 +1870,17 @@
           <t>No (AI TC14 is visual only)</t>
         </is>
       </c>
-      <c r="K18" s="8" t="inlineStr"/>
+      <c r="K18" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
       <c r="L18" s="8" t="inlineStr"/>
-      <c r="M18" s="8" t="inlineStr"/>
+      <c r="M18" s="8" t="inlineStr">
+        <is>
+          <t>DF-05 https://github.com/Toanapr/Homework/issues/5</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1966,7 +2042,11 @@
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr"/>
-      <c r="F5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>Not recorded. No inspection of the cord or plug is in the execution notes.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -1988,7 +2068,11 @@
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Not recorded. TC-14 checked finger access, not whether every clip is engaged.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n">
@@ -2010,7 +2094,11 @@
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>Not recorded. No inspection of the blades for cracks.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -2032,7 +2120,11 @@
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Section 3.1 records a level tiled floor. A clearance of 1 m was not measured.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -2050,11 +2142,19 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>TC-14 / DF-05 was done with the fan unplugged.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -2076,7 +2176,11 @@
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>TC-11 was run by holding the head. The notes do not confirm that the hand stayed on the rear motor housing only.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -2098,7 +2202,11 @@
         </is>
       </c>
       <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr"/>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>Not true of every case. Several executed cases start with the fan already at speed 1 or 2.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -2120,7 +2228,11 @@
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>TC-02 was not run.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -2142,7 +2254,11 @@
         </is>
       </c>
       <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr"/>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>TC-15 was not run. Section 3.1 records about 30 °C for the session, not a reading taken before TC-15.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -2164,7 +2280,11 @@
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>No timed result was recorded. TC-02 and the sweep timing in TC-08 were not completed.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -2186,7 +2306,11 @@
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr"/>
+      <c r="F15" s="8" t="inlineStr">
+        <is>
+          <t>TC-03 was not run.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -2208,7 +2332,11 @@
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>TC-03 was not run.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -2230,7 +2358,11 @@
         </is>
       </c>
       <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr"/>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Tape marks are not mentioned in the TC-08 or TC-13 results. TC-13 was not run.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -2252,7 +2384,11 @@
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>No gap or displacement measurement was recorded. TC-13 was not run.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -2270,11 +2406,19 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="F19" s="8" t="inlineStr">
+        <is>
+          <t>Five YouTube Shorts are linked for TC-06, TC-07, TC-09, TC-10 and TC-12. Shorts are at most 60 s. Narration is the student's own recording.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -2296,7 +2440,11 @@
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr"/>
-      <c r="F20" s="8" t="inlineStr"/>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>Not confirmed from the video links. The model label and date were not checked at the start of each clip.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -2314,11 +2462,19 @@
       </c>
       <c r="D21" s="8" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr"/>
-      <c r="F21" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="F21" s="8" t="inlineStr">
+        <is>
+          <t>The five required videos are Unlisted YouTube Shorts and the links are in the Test Cases sheet. TC-04, TC-08, TC-11 and TC-14 have no video.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -2336,11 +2492,19 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr"/>
-      <c r="F22" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="F22" s="8" t="inlineStr">
+        <is>
+          <t>DF-01 to DF-05 each have a GitHub Issue with steps, expected, actual, severity, impact and the 27/09/2026 observation.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -2358,11 +2522,19 @@
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr"/>
-      <c r="F23" s="8" t="inlineStr"/>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>27/09/2026</t>
+        </is>
+      </c>
+      <c r="F23" s="8" t="inlineStr">
+        <is>
+          <t>Every executed case has an actual result and a verdict. Cases that were not run are marked NOT RUN.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
@@ -2384,7 +2556,11 @@
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr"/>
-      <c r="F24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>TC-01 was not run.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2402,7 +2578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2489,6 +2665,291 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DF-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The fan switches off when the speed knob rests between two marks.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Turn the knob slowly and leave it between two speed marks. Release it and watch for about 10 s.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>The knob snaps to one marked position, or the fan runs steadily at one of the two speeds.</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>When the knob is left between two marks, the fan switches off.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Bedroom, Senko B813, 27/09/2026</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://youtube.com/shorts/k_u6U1VcS8w</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://github.com/Toanapr/Homework/issues/1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DF-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>The motor clicks one beat each time the speed knob passes a midpoint while turning from 1 to 3.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Run the fan at speed 1. Turn the knob in one continuous movement from 1 to 3. Watch the motor each time the pointer passes the midpoint between two marks, then stop on mark 3.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>The speed matches the position the knob stops at, with no stop, hum or stall during the turn.</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Each time the pointer passes the midpoint between two marks, the motor clicks one beat. When the knob stops on a mark, the speed matches that mark.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Bedroom, Senko B813, 27/09/2026</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Observed 27/09/2026 on the Senko B813. No video for this run.</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://github.com/Toanapr/Homework/issues/2</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DF-03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>The head sweeps more than one extra turn after oscillation is switched off.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Run the fan at speed 2 with the head sweeping. Switch the oscillation knob off while the head is still moving. Watch how far the head travels before it stops.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>The head stops within one sweep after oscillation is switched off.</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>After the oscillation knob is switched off while the head is sweeping, the head sweeps more than one extra turn before it stops.</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Bedroom, Senko B813, 27/09/2026</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Observed 27/09/2026 on the Senko B813. No video for this run.</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://github.com/Toanapr/Homework/issues/3</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DF-04</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TC-11</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>The oscillation gear grinds when the head is held, and the head stays still after release.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Run the fan at speed 1 with oscillation on. Hold the head still for 2 seconds, hand on the rear motor housing only. Release the head.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>The gear slips without grinding, and oscillation resumes after the head is released.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>While the head is held, the gears grind. After release the head stays still and oscillation does not resume.</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Bedroom, Senko B813, 27/09/2026</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Observed 27/09/2026 on the Senko B813. No video for this run.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://github.com/Toanapr/Homework/issues/4</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DF-05</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TC-14</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A fingertip can touch a blade through the rear guard.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Unplug the fan and wait until the blades have stopped. Try to touch a blade with a fingertip through the front guard, then through the rear guard.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A fingertip cannot reach a blade through either guard.</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Through the front guard a fingertip cannot touch a blade. Through the rear guard a fingertip can touch a blade.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Bedroom, Senko B813, unplugged, 27/09/2026</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Observed 27/09/2026 on the Senko B813. No video for this run.</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://github.com/Toanapr/Homework/issues/5</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="G5:G40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>